<commit_message>
sent holiday report - removed emoji
</commit_message>
<xml_diff>
--- a/Daily_CSFA_Report.xlsx
+++ b/Daily_CSFA_Report.xlsx
@@ -439,7 +439,7 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🎉 PUBLIC HOLIDAY - Tuesday, February 03, 2026</t>
+          <t xml:space="preserve"> PUBLIC HOLIDAY - Tuesday, February 03, 2026</t>
         </is>
       </c>
     </row>
@@ -449,7 +449,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>No business activities recorded on this date</t>
+          <t>No CSFA activities recorded on this date</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
about to add new changes
</commit_message>
<xml_diff>
--- a/Daily_CSFA_Report.xlsx
+++ b/Daily_CSFA_Report.xlsx
@@ -557,10 +557,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -647,10 +647,10 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -701,10 +701,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="n">
         <v>5</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>1</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -1406,17 +1406,17 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S6" s="5" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>13/20</t>
         </is>
       </c>
     </row>
@@ -1630,17 +1630,17 @@
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S8" s="5" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>9/20</t>
+          <t>6/20</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>14/20</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="25" customHeight="1">
+    <row r="6" ht="39.2" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>INÁCIO RODRIGUES</t>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>No attendance on dates: 16, 17, 18, 19 (4 days)</t>
+          <t>No attendance on dates: 16, 17, 18, 19, 20, 23, 24 (7 days)</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>No attendance on dates: 2, 4, 6, 9, 10, 12, 13, 16, 17, 18, 19 (11 days)</t>
+          <t>No attendance on dates: 2, 4, 6, 9, 10, 12, 13, 16, 17, 18, 19, 20, 23, 24 (14 days)</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="25" customHeight="1">
+    <row r="10" ht="39.2" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>RICARDO MACUACUA</t>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>No attendance on dates: 10, 12, 13, 16, 17 (5 days)</t>
+          <t>No attendance on dates: 10, 12, 13, 16, 17, 23 (6 days)</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -2176,12 +2176,12 @@
     <row r="1" ht="23.6" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>FERRAGEM NHAMPIMBE, EI (visited)</t>
+          <t>FERRAGEM ACACIA (visited)</t>
         </is>
       </c>
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>Time Spent: 00 Hrs 17 Mins</t>
+          <t>Time Spent: 00 Hrs 16 Mins</t>
         </is>
       </c>
       <c r="C1" s="6" t="inlineStr"/>
@@ -2222,102 +2222,66 @@
     <row r="3" ht="39.2" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1025</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>10276 - DILUENTE SINTETICO ECONOMY 5L</t>
+          <t>206-0001-020 - Nation PVA Branco 20L</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="n">
-        <v>5</v>
+        <v>501</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>636</v>
+        <v>1040</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>3,180.00</t>
+          <t>521,040.00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
-    <row r="4" ht="39.2" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>772</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 5L - DARK SERIES</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>1289</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>6,445.00</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="8" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="8" t="n"/>
     </row>
     <row r="5" ht="23.6" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>664</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>PENDLEO TRADE 5L  - DARK SERIES</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>1526.75</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>4,580.25</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM 1º DE MAIO (visited)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 40 Mins</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="23.6" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>PENDLEO TRADE 5L  - 015-001</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>1526.75</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>10,687.25</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="11" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="8" t="n"/>
@@ -2331,12 +2295,12 @@
     <row r="8" ht="23.6" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>SAAK INTERNACIONAL, LDA (visited)</t>
+          <t>CONSTRUA BUILD IT (visited)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Time Spent: 00 Hrs 19 Mins</t>
+          <t>Time Spent: 00 Hrs 27 Mins</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr"/>
@@ -2370,12 +2334,12 @@
     <row r="11" ht="23.6" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>FERRAGEM VAVA, EI (visited)</t>
+          <t>SOLECTRIC, LDA (visited)</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Time Spent: 00 Hrs 25 Mins</t>
+          <t>Time Spent: 00 Hrs 19 Mins</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr"/>
@@ -2406,15 +2370,15 @@
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="8" t="n"/>
     </row>
-    <row r="14" ht="39.2" customHeight="1">
+    <row r="14" ht="23.6" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>OUSAF INTERNATIONAL TRADING LDA (visited)</t>
+          <t>FAZAL COMERCIAL, EI (visited)</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Time Spent: 00 Hrs 17 Mins</t>
+          <t>Time Spent: 00 Hrs 31 Mins</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr"/>
@@ -2445,15 +2409,15 @@
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
     </row>
-    <row r="17" ht="39.2" customHeight="1">
+    <row r="17" ht="23.6" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>ELECTRO FERRAGEM MASTER SOLUTIONS (visited)</t>
+          <t>FERRAGEM COQUEIRO, LDA (visited)</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Time Spent: 00 Hrs 29 Mins</t>
+          <t>Time Spent: 00 Hrs 23 Mins</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr"/>
@@ -2463,315 +2427,215 @@
       <c r="G17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="23.6" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+    </row>
+    <row r="20" ht="39.2" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO DO RIO VERDE, SOC. UNIP. LDA (visited)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 14 Mins</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="23.6" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="39.2" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>FRANCIS FERRAGEM SOC. UNIP. LDA (visited)</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 22 Mins</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr"/>
+      <c r="D23" s="6" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24" ht="23.6" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="11" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+    </row>
+    <row r="26" ht="23.6" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM CHOUPAL (called)</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr"/>
+      <c r="C26" s="6" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr"/>
+      <c r="F26" s="6" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="23.6" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Product ID</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Product Description</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr"/>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr"/>
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Sold Qty</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>Unit Cost</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Order Value</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19" ht="39.2" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>1025</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>10276 - DILUENTE SINTETICO ECONOMY 5L</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="n">
+      <c r="G27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28" ht="23.6" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>GAMMA COR PREMIUM 25KG - 015-001</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E19" s="2" t="n">
-        <v>636</v>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>3,180.00</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20" ht="39.2" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>1024</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>10275 - DILUENTE SINTETICO ECONOMY 1L</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>143</v>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>5,720.00</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
-    </row>
-    <row r="22" ht="23.6" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>FAZAL COMERCIAL, EI (visited)</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 20 Mins</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="6" t="inlineStr"/>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="6" t="inlineStr"/>
-      <c r="G22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="23.6" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="11" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="8" t="n"/>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
-      <c r="G24" s="8" t="n"/>
-    </row>
-    <row r="25" ht="23.6" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM MUNHISSE MNISI, E.I (called)</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr"/>
-      <c r="C25" s="6" t="inlineStr"/>
-      <c r="D25" s="6" t="inlineStr"/>
-      <c r="E25" s="6" t="inlineStr"/>
-      <c r="F25" s="6" t="inlineStr"/>
-      <c r="G25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="23.6" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr"/>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="23.6" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>736</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>PENDAGUA TRADE 20L - DARK SERIES</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>2999.2</v>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>5,998.40</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="8" t="n"/>
-      <c r="B28" s="8" t="n"/>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="n"/>
+      <c r="E28" s="2" t="n">
+        <v>1952.8</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>9,764.00</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="23.6" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM ZAM ZAM (called)</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr"/>
-      <c r="C29" s="6" t="inlineStr"/>
-      <c r="D29" s="6" t="inlineStr"/>
-      <c r="E29" s="6" t="inlineStr"/>
-      <c r="F29" s="6" t="inlineStr"/>
-      <c r="G29" s="6" t="inlineStr"/>
-    </row>
-    <row r="30" ht="23.6" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr"/>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr"/>
-    </row>
-    <row r="31" ht="23.6" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>1023</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>10274 - wallplast  25kgs</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="n">
-        <v>110</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>958</v>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>105,380.00</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32" ht="23.6" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>NATION PVA ECONOMY 20L - 015-001</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="n">
-        <v>501</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>1040</v>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>521,040.00</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="8" t="n"/>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
-      <c r="E33" s="8" t="n"/>
-      <c r="F33" s="8" t="n"/>
-      <c r="G33" s="8" t="n"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>GAMMA COR PREMIUM 25KG - 015-001</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>2244.6</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>6,733.80</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A23:G23"/>
+  <mergeCells count="7">
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A9:G9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2783,7 +2647,1094 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="23.6" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>CONSTRU YAKA (visited)</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 13 Mins</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr"/>
+      <c r="D1" s="6" t="inlineStr"/>
+      <c r="E1" s="6" t="inlineStr"/>
+      <c r="F1" s="6" t="inlineStr"/>
+      <c r="G1" s="6" t="inlineStr"/>
+    </row>
+    <row r="2" ht="23.6" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="11" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="8" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+    </row>
+    <row r="4" ht="23.6" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM ABAB LDA (visited)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 01 Hrs 09 Mins</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="23.6" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="11" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="23.6" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>AKBAR FERRAGEM (visited)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 13 Mins</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="23.6" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="23.6" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>AUTO FERRAGEM LAZARO COME (visited)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 10 Mins</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="23.6" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A11:G11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="23.6" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>TINTAS BERGER MAPUTO OFFICE (visited)</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 18 Mins</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr"/>
+      <c r="D1" s="6" t="inlineStr"/>
+      <c r="E1" s="6" t="inlineStr"/>
+      <c r="F1" s="6" t="inlineStr"/>
+      <c r="G1" s="6" t="inlineStr"/>
+    </row>
+    <row r="2" ht="23.6" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="11" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="8" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+    </row>
+    <row r="4" ht="23.6" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>GIRASSOL TRADING LDA (visited)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 01 Hrs 03 Mins</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="23.6" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6" ht="23.6" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>667</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>CHARME ECONOMY 5L - DARK SERIES</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1320</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>15,840.00</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="23.6" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>CHARME ECONOMY 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1320</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>15,840.00</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="23.6" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>666</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CHARME ECONOMY 1L - DARK SERIES</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>356</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>25,632.00</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="23.6" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CHARME ECONOMY 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>356</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>25,632.00</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="39.2" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ZARCAO SECAGEM NORMAL TRADE 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>386</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>27,792.00</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="23.6" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEIRA SÃO JOSÉ (visited)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 15 Mins</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="23.6" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="23.6" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM INDICO (visited)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 01 Mins</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr"/>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="23.6" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="39.2" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM LABAIK SOC.UNIP, LDA (visited)</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 06 Mins</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="23.6" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+    </row>
+    <row r="21" ht="39.2" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM MACICAME, SOCIEDADE UNIPESSOAL, LDA (visited)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 00 Hrs 53 Mins</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr"/>
+      <c r="D21" s="6" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="23.6" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="23.6" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>4,476.00</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="23.6" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>666</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>CHARME ECONOMY 1L - DARK SERIES</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>364</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>6,552.00</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="23.6" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>CHARME ECONOMY 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>364</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>6,552.00</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="39.2" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>ZARCAO SECAGEM NORMAL TRADE 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>7,092.00</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
+    </row>
+    <row r="28" ht="23.6" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM MUHENGO, LDA (visited)</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 01 Hrs 17 Mins</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29" ht="23.6" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="11" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
+    </row>
+    <row r="31" ht="23.6" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM SERGIO E.I (visited)</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Time Spent: 01 Hrs 32 Mins</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32" ht="23.6" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>No orders</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="11" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+    </row>
+    <row r="34" ht="39.2" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>MAKARAN COMERCIAL-SOCIEDADE UNIPESSOAL, LIMITADA (called)</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr"/>
+      <c r="C34" s="6" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35" ht="23.6" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr"/>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36" ht="23.6" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>SUBCAPA PREMIUM 1L  - 015-001</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>307.35</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>3,073.50</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="39.2" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>1025</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>10276 - DILUENTE SINTETICO ECONOMY 5L</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>636</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>3,180.00</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="39.2" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>ZARCAO SECAGEM NORMAL TRADE 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>7,092.00</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="39.2" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>DILUENTE SINTETICO ECONOMY 0.75L - 015-001</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>3,175.00</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40" ht="23.6" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>1038</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>DILUENTE LAQUER THINNER 750ml</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>3,450.00</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="23.6" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>368</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>8,096.00</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="39.2" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>1030</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>206-0001-020 - Nation PVA Branco 20L</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>1056</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>105,600.00</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+    </row>
+    <row r="44" ht="23.6" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>FERRAGEM RHULANE EI (called)</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr"/>
+      <c r="C44" s="6" t="inlineStr"/>
+      <c r="D44" s="6" t="inlineStr"/>
+      <c r="E44" s="6" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45" ht="23.6" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr"/>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46" ht="23.6" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>3,730.00</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="8" t="n"/>
+      <c r="B47" s="8" t="n"/>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="8" t="n"/>
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -2798,14 +3749,10 @@
     <row r="1" ht="39.2" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>OUSAF INTERNATIONAL TRADING LDA (visited)</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 15 Mins</t>
-        </is>
-      </c>
+          <t>PAIZINHO COMERCIAL SOC. UNIP. LDA (called)</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr"/>
       <c r="C1" s="6" t="inlineStr"/>
       <c r="D1" s="6" t="inlineStr"/>
       <c r="E1" s="6" t="inlineStr"/>
@@ -2813,56 +3760,108 @@
       <c r="G1" s="6" t="inlineStr"/>
     </row>
     <row r="2" ht="23.6" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="11" t="n"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="8" t="n"/>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr"/>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3" ht="39.2" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DILUENTE LAQUER THINNER PREMIUM 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>858</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>17,160.00</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="39.2" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>INDO AFRICA COMERCIAL - ARMAZENS VITORIA (visited)</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 15 Mins</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>193</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>DILUENTE LAQUER THINNER PREMIUM 1L -015-001</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>205</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>20,500.00</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="23.6" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="11" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 20L - 015-001</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>104,000.00</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="n"/>
@@ -2876,14 +3875,10 @@
     <row r="7" ht="23.6" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>FARZANA SERVICES (visited)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 15 Mins</t>
-        </is>
-      </c>
+          <t>TINTAS E FERRAGENS, LDA (called)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr"/>
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr"/>
@@ -2891,94 +3886,130 @@
       <c r="G7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="23.6" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="11" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr"/>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="39.2" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>1021</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>10272 - CORANTE CROWN DU T MEDIUM 1L</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1671.24</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>40,109.76</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="39.2" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM - E- HUSSAIN SOC. UNIP LDA - AV. JOSINA MACHEL. BAIXA (visited)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 35 Mins</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="6" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="23.6" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr"/>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>10263 - CORANTE CROWN DU AXX ORGANIC 1L</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1364.72</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>16,376.64</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="39.2" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1018</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>10269 - CORANTE CROWN DU QS HS YELLOW 1L</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>2201.59</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>26,419.08</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="39.2" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 1L - 015-001</t>
+          <t>10259 - CORANTE CROWN DU C YELLOW 1L</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>325</v>
+        <v>902.85</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>3,250.00</t>
+          <t>21,668.40</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -2986,278 +4017,374 @@
     <row r="13" ht="39.2" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>1017</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 1L - DARK SERIES</t>
+          <t>10268 - CORANTE CROWN DU V MAGENTA 1L</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>325</v>
+        <v>1483.32</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>3,250.00</t>
+          <t>26,699.76</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
-    <row r="14" ht="23.6" customHeight="1">
+    <row r="14" ht="39.2" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>1007</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHARME ECONOMY 5L - 015-001</t>
+          <t>10258 - CORANTE CROWN DU B  BLACK 1L</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1333</v>
+        <v>663.15</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>13,330.00</t>
+          <t>15,915.60</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
-    <row r="15" ht="23.6" customHeight="1">
+    <row r="15" ht="39.2" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>NATION PVA ECONOMY 5L - 015-001</t>
+          <t>10260 - CORANTE CROWN DU F RED OXIDE 1L</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>373</v>
+        <v>1008</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>3,730.00</t>
+          <t>18,144.00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
-    <row r="16" ht="23.6" customHeight="1">
+    <row r="16" ht="39.2" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>1010</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>PREMIER PREMIUM 20L -015-001</t>
+          <t>10261 - CORANTE CROWN DU XX WHITE 1L</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1122.51</v>
+        <v>983.87</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>11,225.10</t>
+          <t>17,709.66</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
-    <row r="17" ht="23.6" customHeight="1">
+    <row r="17" ht="39.2" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1014</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>NATION PVA ECONOMY 20L - 015-001</t>
+          <t>10265 - CORANTE CROWN DU E PHTHALO 1L</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>748.34</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>13,470.12</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="39.2" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>937</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>081-1001 - PENDAGUA PASTEL BASE 20L</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>2105.54</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>21,055.40</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="23.6" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>938</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>081-1002 - PENDAGUA DEEP BASE 20L</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1993.62</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>29,904.30</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="39.2" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>960</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>10211 - SILKY SMOOTH PASTEL BASE 5L</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>925.4</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>18,508.00</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="39.2" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>928</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>119-1001 - SILKY SMOOTH PASTEL BASE 20L</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="E17" s="2" t="n">
-        <v>1088</v>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>27,200.00</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="8" t="n"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="8" t="n"/>
-      <c r="G18" s="8" t="n"/>
-    </row>
-    <row r="19" ht="23.6" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>ARIMEK COMERCIAL EI (visited)</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 20 Mins</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr"/>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="23.6" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="11" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
+      <c r="E21" s="2" t="n">
+        <v>3279.48</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>81,987.00</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
     </row>
     <row r="22" ht="39.2" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>MBFL FERRAGENS - SOC. UNIP. LDA (visited)</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 15 Mins</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="6" t="inlineStr"/>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="6" t="inlineStr"/>
-      <c r="G22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="23.6" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="11" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="8" t="n"/>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
-      <c r="G24" s="8" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>964</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>10215 - SILKY SMOOTH ACCENT BASE 5L</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1060.24</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>26,506.00</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="39.2" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>119-1003 - SILKY SMOOTH ACCENT BASE 20L</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>3866.28</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>96,657.00</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="23.6" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>962</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>10213 - SILKY SMOOTH DEEP BASE 5L</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>876.12</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>13,141.80</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="39.2" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM HUSSAIN E.I AV ANGOLA 2216 (called)</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr"/>
-      <c r="C25" s="6" t="inlineStr"/>
-      <c r="D25" s="6" t="inlineStr"/>
-      <c r="E25" s="6" t="inlineStr"/>
-      <c r="F25" s="6" t="inlineStr"/>
-      <c r="G25" s="6" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>929</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>119-1002 - SILKY SMOOTH DEEP BASE 20L</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>3142.86</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>157,143.00</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
     </row>
     <row r="26" ht="23.6" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr"/>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="39.2" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>SILKY SMOOTH PREMIUM 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>1098</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>16,470.00</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="23.6" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>83</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 1L - 015-001</t>
+          <t>SILKY SMOOTH PREMIUM 20L - 015-001</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>325</v>
+        <v>3256</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>3,250.00</t>
+          <t>48,840.00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -3265,24 +4392,24 @@
     <row r="28" ht="39.2" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 1L - DARK SERIES</t>
+          <t>CROWN ECO VESTA ECONOMY 20L - 015-001</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>325</v>
+        <v>1333</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>3,250.00</t>
+          <t>33,325.00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
@@ -3290,933 +4417,591 @@
     <row r="29" ht="23.6" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>667</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>CHARME ECONOMY 5L - 015-001</t>
+          <t>CHARME ECONOMY 5L - DARK SERIES</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1333</v>
+        <v>1320</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>13,330.00</t>
+          <t>19,800.00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
-    <row r="30" ht="39.2" customHeight="1">
+    <row r="30" ht="23.6" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>NATION ESMALTE ECONOMY 5L - 015-001</t>
+          <t>CHARME ECONOMY 1L - 015-001</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>3,730.00</t>
+          <t>5,460.00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
-    <row r="31" ht="39.2" customHeight="1">
+    <row r="31" ht="23.6" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>666</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>NATION ESMALTE ECONOMY 20L - 015-001</t>
+          <t>CHARME ECONOMY 1L - DARK SERIES</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>1088</v>
+        <v>364</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>27,200.00</t>
+          <t>5,460.00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="8" t="n"/>
-      <c r="B32" s="8" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="n"/>
-      <c r="F32" s="8" t="n"/>
-      <c r="G32" s="8" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A23:G23"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="23.6" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>TINTAS BERGER MAPUTO OFFICE (visited)</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 48 Mins</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr"/>
-      <c r="D1" s="6" t="inlineStr"/>
-      <c r="E1" s="6" t="inlineStr"/>
-      <c r="F1" s="6" t="inlineStr"/>
-      <c r="G1" s="6" t="inlineStr"/>
-    </row>
-    <row r="2" ht="23.6" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="11" t="n"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="8" t="n"/>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-    </row>
-    <row r="4" ht="23.6" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>ELECTRO FERRAGEM BIÉ,E.I (visited)</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 17 Mins</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="23.6" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="11" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-    </row>
-    <row r="7" ht="39.2" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>MAKARAN COMERCIAL-SOCIEDADE UNIPESSOAL, LIMITADA (visited)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 17 Mins</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="23.6" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="11" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-    </row>
-    <row r="10" ht="23.6" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>SOHA TRADING. SOC. UNIP (visited)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 03 Mins</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="6" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="23.6" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr"/>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="23.6" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="32" ht="23.6" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>NATION PVA ECONOMY 5L - 015-001</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>368</v>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>11,040.00</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-    </row>
-    <row r="14" ht="23.6" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>SUGIRA FERRAGEM, SU,LDA (visited)</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 37 Mins</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr"/>
-      <c r="D14" s="6" t="inlineStr"/>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="23.6" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="11" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="8" t="n"/>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
-    </row>
-    <row r="17" ht="39.2" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM MACICAME, SOCIEDADE UNIPESSOAL, LDA (visited)</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 42 Mins</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr"/>
-      <c r="D17" s="6" t="inlineStr"/>
-      <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="6" t="inlineStr"/>
-      <c r="G17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18" ht="23.6" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="11" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
-    </row>
-    <row r="20" ht="39.2" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>NAWAZ TRADER, COMERCIAL. SOC. UNIP.LDA (visited)</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 16 Mins</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr"/>
-      <c r="D20" s="6" t="inlineStr"/>
-      <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="23.6" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="11" t="n"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="8" t="n"/>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="n"/>
-    </row>
-    <row r="23" ht="23.6" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>CUAMBA&amp;#039;S FERRAGEM, EI (visited)</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 56 Mins</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr"/>
-      <c r="D23" s="6" t="inlineStr"/>
-      <c r="E23" s="6" t="inlineStr"/>
-      <c r="F23" s="6" t="inlineStr"/>
-      <c r="G23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24" ht="23.6" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="11" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="n"/>
-    </row>
-    <row r="26" ht="23.6" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM YANG, SU,LDA (called)</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr"/>
-      <c r="C26" s="6" t="inlineStr"/>
-      <c r="D26" s="6" t="inlineStr"/>
-      <c r="E26" s="6" t="inlineStr"/>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="23.6" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="39.2" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>ZARCAO SECAGEM NORMAL TRADE 1L - 015-001</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="n">
-        <v>108</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>386</v>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>41,688.00</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="8" t="n"/>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="8" t="n"/>
-      <c r="G29" s="8" t="n"/>
-    </row>
-    <row r="30" ht="23.6" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM RHULANE EI (called)</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr"/>
-      <c r="C30" s="6" t="inlineStr"/>
-      <c r="D30" s="6" t="inlineStr"/>
-      <c r="E30" s="6" t="inlineStr"/>
-      <c r="F30" s="6" t="inlineStr"/>
-      <c r="G30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="23.6" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr"/>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr"/>
-    </row>
-    <row r="32" ht="39.2" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>1030</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>206-0001-020 - Nation PVA Branco 20L</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1088</v>
+        <v>368</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>23,936.00</t>
+          <t>18,400.00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="8" t="n"/>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
-      <c r="E33" s="8" t="n"/>
-      <c r="F33" s="8" t="n"/>
-      <c r="G33" s="8" t="n"/>
+    <row r="33" ht="23.6" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 20L - 015-001</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>104,000.00</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34" ht="39.2" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>ZARCAO SECAGEM NORMAL TRADE 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>5,910.00</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="n"/>
+    </row>
+    <row r="36" ht="39.2" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>COMPANHIA DONA CECILIA FERRAGEM (called)</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="23.6" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr"/>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr"/>
+    </row>
+    <row r="38" ht="23.6" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 20L - 015-001</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>520,000.00</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+    </row>
+    <row r="40" ht="23.6" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>ELECTRO FERRAGEM NDZIMANE LDA (called)</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr"/>
+      <c r="C40" s="6" t="inlineStr"/>
+      <c r="D40" s="6" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr"/>
+      <c r="F40" s="6" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41" ht="23.6" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr"/>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42" ht="23.6" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 20L - 015-001</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>156,000.00</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="39.2" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>DILUENTE SINTETICO ECONOMY 0.75L - 015-001</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>9,300.00</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="23.6" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>3,730.00</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="8" t="n"/>
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="8" t="n"/>
+    </row>
+    <row r="46" ht="23.6" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>P.P. IMPORTACAO E EXPORTACAO (called)</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr"/>
+      <c r="C46" s="6" t="inlineStr"/>
+      <c r="D46" s="6" t="inlineStr"/>
+      <c r="E46" s="6" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr"/>
+      <c r="G46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47" ht="23.6" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr"/>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Sold Qty</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Order Value</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr"/>
+    </row>
+    <row r="48" ht="39.2" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>769</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 0.5L - DARK SERIES</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>188.55</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>13,575.60</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="23.6" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>CHARME ECONOMY 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>1428.57</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>7,142.85</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50" ht="39.2" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>771</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 1L - DARK SERIES</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>478.67</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>19,146.80</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="39.2" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 1L - 015-001</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr"/>
+      <c r="D51" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>344.64</v>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>20,678.40</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52" ht="39.2" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 0.5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>188.55</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>20,363.40</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="23.6" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 5L - 015-001</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>377.97</v>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>9,449.25</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="23.6" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>NATION PVA ECONOMY 20L - 015-001</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>1039.5</v>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>155,925.00</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A5:G5"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="23.6" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>TINTAS E FERRAGENS, LDA (visited)</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 53 Mins</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr"/>
-      <c r="D1" s="6" t="inlineStr"/>
-      <c r="E1" s="6" t="inlineStr"/>
-      <c r="F1" s="6" t="inlineStr"/>
-      <c r="G1" s="6" t="inlineStr"/>
-    </row>
-    <row r="2" ht="23.6" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="11" t="n"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="8" t="n"/>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-    </row>
-    <row r="4" ht="23.6" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>P.P. IMPORTACAO E EXPORTACAO (visited)</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 15 Mins</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="23.6" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="11" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-    </row>
-    <row r="7" ht="23.6" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>NATVARLAL COMERCIAL EI (visited)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 41 Mins</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="23.6" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="11" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-    </row>
-    <row r="10" ht="23.6" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>ABDUL SULTANE (visited)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 11 Mins</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="6" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="23.6" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="11" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="23.6" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>FERRAGEM GUAMBE (visited)</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Time Spent: 00 Hrs 23 Mins</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr"/>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="23.6" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>No orders</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="11" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="8" t="n"/>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
-    </row>
-    <row r="16" ht="23.6" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>DAFITI COMERCIO E SERVICO LDA (called)</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr"/>
-      <c r="C16" s="6" t="inlineStr"/>
-      <c r="D16" s="6" t="inlineStr"/>
-      <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17" ht="23.6" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Product Description</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr"/>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Sold Qty</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Unit Cost</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Order Value</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr"/>
-    </row>
-    <row r="18" ht="39.2" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>126</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>VERNIZ PARA MADEIRA INCOLOR+ CORES PREMIUM 1L - 015-001</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>328.23</v>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>6,564.60</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A5:G5"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
works, but be careful with emails
</commit_message>
<xml_diff>
--- a/Daily_CSFA_Report.xlsx
+++ b/Daily_CSFA_Report.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Day Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Attendance Grid - February" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Monthly Attendance - February" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Day Visits" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -870,19 +871,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T2" s="4" t="inlineStr"/>
+      <c r="U2" s="4" t="inlineStr"/>
       <c r="V2" s="4" t="inlineStr">
         <is>
-          <t>20/20 - Perfect attendance</t>
+          <t>18/18 - Perfect attendance</t>
         </is>
       </c>
     </row>
@@ -982,19 +975,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T3" s="4" t="inlineStr"/>
+      <c r="U3" s="4" t="inlineStr"/>
       <c r="V3" s="4" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>17/18</t>
         </is>
       </c>
     </row>
@@ -1094,19 +1079,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T4" s="4" t="inlineStr"/>
+      <c r="U4" s="4" t="inlineStr"/>
       <c r="V4" s="4" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>15/18</t>
         </is>
       </c>
     </row>
@@ -1206,19 +1183,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
+      <c r="T5" s="4" t="inlineStr"/>
+      <c r="U5" s="4" t="inlineStr"/>
       <c r="V5" s="4" t="inlineStr">
         <is>
-          <t>0/20</t>
+          <t>0/18</t>
         </is>
       </c>
     </row>
@@ -1318,19 +1287,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T6" s="4" t="inlineStr"/>
+      <c r="U6" s="4" t="inlineStr"/>
       <c r="V6" s="4" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>10/18</t>
         </is>
       </c>
     </row>
@@ -1430,19 +1391,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T7" s="4" t="inlineStr"/>
+      <c r="U7" s="4" t="inlineStr"/>
       <c r="V7" s="4" t="inlineStr">
         <is>
-          <t>20/20 - Perfect attendance</t>
+          <t>18/18 - Perfect attendance</t>
         </is>
       </c>
     </row>
@@ -1542,19 +1495,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T8" s="4" t="inlineStr"/>
+      <c r="U8" s="4" t="inlineStr"/>
       <c r="V8" s="4" t="inlineStr">
         <is>
-          <t>5/20</t>
+          <t>3/18</t>
         </is>
       </c>
     </row>
@@ -1654,19 +1599,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T9" s="4" t="inlineStr"/>
+      <c r="U9" s="4" t="inlineStr"/>
       <c r="V9" s="4" t="inlineStr">
         <is>
-          <t>20/20 - Perfect attendance</t>
+          <t>18/18 - Perfect attendance</t>
         </is>
       </c>
     </row>
@@ -1766,19 +1703,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T10" s="4" t="inlineStr"/>
+      <c r="U10" s="4" t="inlineStr"/>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>10/18</t>
         </is>
       </c>
     </row>
@@ -1878,19 +1807,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T11" s="4" t="inlineStr"/>
+      <c r="U11" s="4" t="inlineStr"/>
       <c r="V11" s="4" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>15/18</t>
         </is>
       </c>
     </row>
@@ -2047,4 +1968,465 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Salesperson</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Customer Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Time Spent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ANDRE MARQUEZA</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM NHAMPIMBE, EI</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 56 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ANDRE MARQUEZA</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>TELLES COMERCIO &amp;amp; SERVICOS, LDA.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 21 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ANDRE MARQUEZA</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FUXIN MATERIAL DE CONSTRUCAO TRADING, LDA</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 33 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ANDRE MARQUEZA</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ELECTRO FERRAGEM AFRICA, LDA</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 43 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ANDRE MARQUEZA</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>FIVE STAR COMERCIAL, EI</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 31 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ANDRE MARQUEZA</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM MAHNOOR</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 21 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ANDRE MARQUEZA</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM PONTE, LDA</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 41 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM TREVO FAMILIA</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 16 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM ALEX UCUCHO87</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 17 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ELETRICA VOLTZ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 17 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>HOME STORE</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 17 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>AQUAPESCA</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 17 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>KINTECH INTERNATIONAL CO SOCIEDADE UNIPESSOAL,LDA</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 19 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>ITO BENEDITO</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM LIU</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 06 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ITO BENEDITO</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM ZAINAB, LDA</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 15 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ITO BENEDITO</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM DA PRACA</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 19 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ITO BENEDITO</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>MACOMAT MAT. CONSTRUCAO DE MOC.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 03 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ITO BENEDITO</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>GOD WIN FERRAGEM</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 20 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ITO BENEDITO</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM PURE ON HEART</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 12 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ITO BENEDITO</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>BLESSED MIKO IMPORT AND EXPORT, EI</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 00 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>TINTAS BERGER MAPUTO OFFICE</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 00 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>TINTAS BERGER MAPUTO OFFICE</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 45 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>AF FERRAGEM E.I</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 27 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEIRA SÃO JOSÉ</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 38 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM YANG, SU,LDA</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 31 Mins</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added suspensions & new users tracking
</commit_message>
<xml_diff>
--- a/Daily_CSFA_Report.xlsx
+++ b/Daily_CSFA_Report.xlsx
@@ -42,7 +42,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
         <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -82,10 +88,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -453,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -481,11 +493,11 @@
     <row r="2" ht="23.6" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -496,11 +508,11 @@
     <row r="3" ht="23.6" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -511,56 +523,56 @@
     <row r="4" ht="23.6" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Used App</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="23.6" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
           <t>HENRIQUE BERTUR</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Did Not Use App</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="23.6" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>IMRAN AHMED</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Used App</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Suspended</t>
         </is>
       </c>
     </row>
     <row r="6" ht="23.6" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>IMRAN AHMED</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Used App</t>
+          <t>Did Not Use App</t>
         </is>
       </c>
     </row>
     <row r="7" ht="23.6" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -571,11 +583,11 @@
     <row r="8" ht="23.6" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -586,28 +598,43 @@
     <row r="9" ht="23.6" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Used App</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="23.6" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>RICARDO MACUACUA</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Did Not Use App</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="23.6" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Suspended</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="23.6" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>SAIDATA ZALIA</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Used App</t>
         </is>
@@ -624,7 +651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -650,7 +677,7 @@
     <col width="4" customWidth="1" min="21" max="21"/>
     <col width="4" customWidth="1" min="22" max="22"/>
     <col width="4" customWidth="1" min="23" max="23"/>
-    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="35" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -776,776 +803,850 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>ADERITO MACHOVO</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr"/>
+      <c r="C2" s="5" t="inlineStr"/>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr"/>
+      <c r="I2" s="5" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr"/>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr"/>
+      <c r="Q2" s="5" t="inlineStr"/>
+      <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" s="5" t="inlineStr"/>
+      <c r="T2" s="5" t="inlineStr"/>
+      <c r="U2" s="5" t="inlineStr"/>
+      <c r="V2" s="5" t="inlineStr"/>
+      <c r="W2" s="5" t="inlineStr"/>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>1/1 - Perfect attendance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>ANDRE MARQUEZA</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr"/>
-      <c r="P2" s="4" t="inlineStr"/>
-      <c r="Q2" s="4" t="inlineStr"/>
-      <c r="R2" s="4" t="inlineStr"/>
-      <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
-      <c r="V2" s="4" t="inlineStr"/>
-      <c r="W2" s="4" t="inlineStr"/>
-      <c r="X2" s="4" t="inlineStr">
-        <is>
-          <t>12/13</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr"/>
+      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr"/>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>FRANCISCO TOMAS</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
-      <c r="Q3" s="4" t="inlineStr"/>
-      <c r="R3" s="4" t="inlineStr"/>
-      <c r="S3" s="4" t="inlineStr"/>
-      <c r="T3" s="4" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr"/>
-      <c r="V3" s="4" t="inlineStr"/>
-      <c r="W3" s="4" t="inlineStr"/>
-      <c r="X3" s="4" t="inlineStr">
-        <is>
-          <t>12/13</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr"/>
+      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" s="5" t="inlineStr"/>
+      <c r="T4" s="5" t="inlineStr"/>
+      <c r="U4" s="5" t="inlineStr"/>
+      <c r="V4" s="5" t="inlineStr"/>
+      <c r="W4" s="5" t="inlineStr"/>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>HENRIQUE BERTUR</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr"/>
-      <c r="P4" s="4" t="inlineStr"/>
-      <c r="Q4" s="4" t="inlineStr"/>
-      <c r="R4" s="4" t="inlineStr"/>
-      <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr"/>
-      <c r="V4" s="4" t="inlineStr"/>
-      <c r="W4" s="4" t="inlineStr"/>
-      <c r="X4" s="4" t="inlineStr">
-        <is>
-          <t>8/13</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr"/>
+      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" s="5" t="inlineStr"/>
+      <c r="T5" s="5" t="inlineStr"/>
+      <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5" s="5" t="inlineStr"/>
+      <c r="W5" s="5" t="inlineStr"/>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>8/13 | Suspended from 2026-03-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>IMRAN AHMED</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
-      <c r="Q5" s="4" t="inlineStr"/>
-      <c r="R5" s="4" t="inlineStr"/>
-      <c r="S5" s="4" t="inlineStr"/>
-      <c r="T5" s="4" t="inlineStr"/>
-      <c r="U5" s="4" t="inlineStr"/>
-      <c r="V5" s="4" t="inlineStr"/>
-      <c r="W5" s="4" t="inlineStr"/>
-      <c r="X5" s="4" t="inlineStr">
-        <is>
-          <t>6/13</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr"/>
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="5" t="inlineStr"/>
+      <c r="U6" s="5" t="inlineStr"/>
+      <c r="V6" s="5" t="inlineStr"/>
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>6/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>ITO BENEDITO</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
-      <c r="Q6" s="4" t="inlineStr"/>
-      <c r="R6" s="4" t="inlineStr"/>
-      <c r="S6" s="4" t="inlineStr"/>
-      <c r="T6" s="4" t="inlineStr"/>
-      <c r="U6" s="4" t="inlineStr"/>
-      <c r="V6" s="4" t="inlineStr"/>
-      <c r="W6" s="4" t="inlineStr"/>
-      <c r="X6" s="4" t="inlineStr">
-        <is>
-          <t>13/13 - Perfect attendance</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr"/>
+      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr"/>
+      <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="5" t="inlineStr"/>
+      <c r="U7" s="5" t="inlineStr"/>
+      <c r="V7" s="5" t="inlineStr"/>
+      <c r="W7" s="5" t="inlineStr"/>
+      <c r="X7" s="5" t="inlineStr">
+        <is>
+          <t>14/14 - Perfect attendance</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
-      <c r="Q7" s="4" t="inlineStr"/>
-      <c r="R7" s="4" t="inlineStr"/>
-      <c r="S7" s="4" t="inlineStr"/>
-      <c r="T7" s="4" t="inlineStr"/>
-      <c r="U7" s="4" t="inlineStr"/>
-      <c r="V7" s="4" t="inlineStr"/>
-      <c r="W7" s="4" t="inlineStr"/>
-      <c r="X7" s="4" t="inlineStr">
-        <is>
-          <t>12/13</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr"/>
+      <c r="Q8" s="5" t="inlineStr"/>
+      <c r="R8" s="5" t="inlineStr"/>
+      <c r="S8" s="5" t="inlineStr"/>
+      <c r="T8" s="5" t="inlineStr"/>
+      <c r="U8" s="5" t="inlineStr"/>
+      <c r="V8" s="5" t="inlineStr"/>
+      <c r="W8" s="5" t="inlineStr"/>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>RICARDO DINIS LANGA</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr"/>
-      <c r="P8" s="4" t="inlineStr"/>
-      <c r="Q8" s="4" t="inlineStr"/>
-      <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr"/>
-      <c r="T8" s="4" t="inlineStr"/>
-      <c r="U8" s="4" t="inlineStr"/>
-      <c r="V8" s="4" t="inlineStr"/>
-      <c r="W8" s="4" t="inlineStr"/>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>13/13 - Perfect attendance</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr"/>
+      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" s="5" t="inlineStr"/>
+      <c r="T9" s="5" t="inlineStr"/>
+      <c r="U9" s="5" t="inlineStr"/>
+      <c r="V9" s="5" t="inlineStr"/>
+      <c r="W9" s="5" t="inlineStr"/>
+      <c r="X9" s="5" t="inlineStr">
+        <is>
+          <t>14/14 - Perfect attendance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>RICARDO MACUACUA</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr"/>
+      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" s="5" t="inlineStr"/>
+      <c r="T10" s="5" t="inlineStr"/>
+      <c r="U10" s="5" t="inlineStr"/>
+      <c r="V10" s="5" t="inlineStr"/>
+      <c r="W10" s="5" t="inlineStr"/>
+      <c r="X10" s="5" t="inlineStr">
+        <is>
+          <t>10/12 | Suspended from 2026-03-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>SAIDATA ZALIA</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
-      <c r="Q9" s="4" t="inlineStr"/>
-      <c r="R9" s="4" t="inlineStr"/>
-      <c r="S9" s="4" t="inlineStr"/>
-      <c r="T9" s="4" t="inlineStr"/>
-      <c r="U9" s="4" t="inlineStr"/>
-      <c r="V9" s="4" t="inlineStr"/>
-      <c r="W9" s="4" t="inlineStr"/>
-      <c r="X9" s="4" t="inlineStr">
-        <is>
-          <t>10/13</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>SAIDATA ZALIA</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="4" t="inlineStr"/>
-      <c r="Q10" s="4" t="inlineStr"/>
-      <c r="R10" s="4" t="inlineStr"/>
-      <c r="S10" s="4" t="inlineStr"/>
-      <c r="T10" s="4" t="inlineStr"/>
-      <c r="U10" s="4" t="inlineStr"/>
-      <c r="V10" s="4" t="inlineStr"/>
-      <c r="W10" s="4" t="inlineStr"/>
-      <c r="X10" s="4" t="inlineStr">
-        <is>
-          <t>9/13</t>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="R11" s="5" t="inlineStr"/>
+      <c r="S11" s="5" t="inlineStr"/>
+      <c r="T11" s="5" t="inlineStr"/>
+      <c r="U11" s="5" t="inlineStr"/>
+      <c r="V11" s="5" t="inlineStr"/>
+      <c r="W11" s="5" t="inlineStr"/>
+      <c r="X11" s="5" t="inlineStr">
+        <is>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1582,106 +1683,118 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Perfect attendance</t>
+          <t>New starter from 2026-03-19</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>No attendance on date: 16</t>
+          <t>Perfect attendance</t>
         </is>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>FRANCISCO TOMAS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>No attendance on date: 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39.2" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
           <t>HENRIQUE BERTUR</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>No attendance on dates: 2, 4, 10, 11, 18 (5 days)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>IMRAN AHMED</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>No attendance on dates: 4, 5, 6, 9, 11 (5 days)</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>No attendance on dates: 2, 4, 10, 11, 18 (5 days) | Suspended from 2026-03-19</t>
         </is>
       </c>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>IMRAN AHMED</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Perfect attendance</t>
+          <t>No attendance on dates: 4, 5, 6, 9, 11, 19 (6 days)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>No attendance on date: 2</t>
+          <t>Perfect attendance</t>
         </is>
       </c>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Perfect attendance</t>
+          <t>No attendance on date: 2</t>
         </is>
       </c>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Perfect attendance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="39.2" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>RICARDO MACUACUA</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>No attendance on dates: 2, 3, 18 (3 days)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>No attendance on dates: 2, 3, 18 (3 days) | Suspended from 2026-03-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>SAIDATA ZALIA</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>No attendance on dates: 2, 3, 4, 13 (4 days)</t>
         </is>
@@ -1698,7 +1811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1726,352 +1839,352 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MALABAR MATERIAL DE CONSTRUCAO SOCIEDADE UNIPESSOAL, LD</t>
+          <t>MAGUENGUE AUTO-PAINTS</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 28 Mins</t>
+          <t>00 Hrs 16 Mins</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM SABHA, LDA</t>
+          <t>UAMUSSE FERRANGEM</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 35 Mins</t>
+          <t>00 Hrs 07 Mins</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM MAHNOOR</t>
+          <t>FERRAGEM GLORIOSO</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 46 Mins</t>
+          <t>00 Hrs 15 Mins</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>FUXIN MATERIAL DE CONSTRUCAO TRADING, LDA</t>
+          <t>ROYAL FERRAGEM SUCURSAL LDA</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 30 Mins</t>
+          <t>00 Hrs 10 Mins</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM ACACIA</t>
+          <t>FERRAGEM UNIVERSAL</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>01 Hrs 02 Mins</t>
+          <t>00 Hrs 08 Mins</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM ZINTAVA SOC UNP LDA</t>
+          <t>P.P. IMPORTACAO E EXPORTACAO</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 45 Mins</t>
+          <t>00 Hrs 08 Mins</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>R.V ELECTRO FERRAGEM LDA</t>
+          <t>LANGA COMERCIAL SOC UNP LDA</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 00 Mins</t>
+          <t>00 Hrs 08 Mins</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM TREVO FAMILIA</t>
+          <t>FERRAGEM TENHA FÉ</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 06 Mins</t>
+          <t>00 Hrs 08 Mins</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ADERITO MACHOVO</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM ALEX UCUCHO87</t>
+          <t>TINTAS E FERRAGENS, LDA</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 06 Mins</t>
+          <t>00 Hrs 07 Mins</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM FORTALEZA</t>
+          <t>MASSANGO PAINTS, EI</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 10 Mins</t>
+          <t>00 Hrs 17 Mins</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SSR TRADING</t>
+          <t>FERRAGEM DAS MAHOTAS,LDA</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 15 Mins</t>
+          <t>00 Hrs 21 Mins</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>GODS PLAN</t>
+          <t>QUATRO ESTRELAS FERRAGENS</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>01 Hrs 03 Mins</t>
+          <t>00 Hrs 43 Mins</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM LANGA</t>
+          <t>CHINA MALL, LDA</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 19 Mins</t>
+          <t>00 Hrs 30 Mins</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>IMRAN AHMED</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>NOSSA FERRAGEM SOCIEDADE UNIPESSOAL LIMITADA</t>
+          <t>KUSHI MAPUTO LDA</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 07 Mins</t>
+          <t>00 Hrs 16 Mins</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>IMRAN AHMED</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>LBN COMERCIAL,LDA</t>
+          <t>FERRAGEM PONTE, LDA</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 27 Mins</t>
+          <t>00 Hrs 16 Mins</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>IMRAN AHMED</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM ALAR,LDA</t>
+          <t>LIMPOPO TRADING, LDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 12 Mins</t>
+          <t>00 Hrs 29 Mins</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>IMRAN AHMED</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM ERA , NAMPULA</t>
+          <t>FERRAGEM CH CONSTRUCOES</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 19 Mins</t>
+          <t>00 Hrs 15 Mins</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>IMRAN AHMED</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>BLUE OCEAN, LIMITADA ( SUCURSAL) NAMPULA</t>
+          <t>FERRAGEM SOBRINHO DE DEUS</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 10 Mins</t>
+          <t>00 Hrs 08 Mins</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM JAIME ELIAS MABOXE</t>
+          <t>PATEL HARDWARE MOCAMBIQUE</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 33 Mins</t>
+          <t>00 Hrs 09 Mins</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>J. ELECTRO FERRAGEM SOC. UNIP. LDA</t>
+          <t>FERRAGEM RHUMBANE</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 11 Mins</t>
+          <t>00 Hrs 15 Mins</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>BLESSED MIKO IMPORT AND EXPORT, EI</t>
+          <t>JIANGHAI CONSTRUCOES E SOCIEDADE UNIPESSOAL, LDA</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2083,357 +2196,459 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>HENRIQUE BERTUR</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM SORTHIA, LDA</t>
+          <t>KULUN MATERIAL DE CONSTRUCAO, LIMITADA</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 09 Mins</t>
+          <t>00 Hrs 25 Mins</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>HENRIQUE BERTUR</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>MFD FERRAGEM</t>
+          <t>FERCON</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 06 Mins</t>
+          <t>00 Hrs 24 Mins</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>HENRIQUE BERTUR</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM KULSOOM LDA</t>
+          <t>FERRAGEM MAHAMCOMERCIAL</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 05 Mins</t>
+          <t>00 Hrs 02 Mins</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>HENRIQUE BERTUR</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM DA PRACA</t>
+          <t>ROSE GONSALVES</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 04 Mins</t>
+          <t>00 Hrs 25 Mins</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>HENRIQUE BERTUR</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM MUIZ, EI</t>
+          <t>HAO FA COMERCIAL</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 14 Mins</t>
+          <t>01 Hrs 18 Mins</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>HENRIQUE BERTUR</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>HOTEL RANIS</t>
+          <t>FERNEX FERRAGEM</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 18 Mins</t>
+          <t>00 Hrs 05 Mins</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>HENRIQUE BERTUR</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>CONSTRUA MEHEK</t>
+          <t>IMRAN FERRAGEM</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 04 Mins</t>
+          <t>00 Hrs 16 Mins</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>KULUN MATERIAL DE CONSTRUCAO</t>
+          <t>FERRAGEM AFRIPAK TRADING EI</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 06 Mins</t>
+          <t>00 Hrs 09 Mins</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>FERCON</t>
+          <t>ARIMEK COMERCIAL EI</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 08 Mins</t>
+          <t>00 Hrs 18 Mins</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>KEYU COMERCIAL</t>
+          <t>MODALAND INTERPRICES</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 07 Mins</t>
+          <t>00 Hrs 09 Mins</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>KUMAR CHAMPAKLAL</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>FORMEX MOCAMBIQUE BAIXA</t>
+          <t>GOD WIN FERRAGEM</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 07 Mins</t>
+          <t>00 Hrs 06 Mins</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>TINTAS BERGER MAPUTO OFFICE</t>
+          <t>FERRAGEM AUTO GEMO</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 18 Mins</t>
+          <t>00 Hrs 05 Mins</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>SIMBA HOME CARE, SU,LDA</t>
+          <t>MOBILITY INVESTIMENTO, EI</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 21 Mins</t>
+          <t>00 Hrs 14 Mins</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEIRA SÃO JOSÉ</t>
+          <t>FERRAGEM PURE ON HEART</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 23 Mins</t>
+          <t>00 Hrs 03 Mins</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>NELITO SIMANGO INVESTIMENTO, SU,LDA</t>
+          <t>LUA E MAR</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 28 Mins</t>
+          <t>00 Hrs 47 Mins</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>AC CHARLES - SOCIEDADE UNIPESSOAL, LDA</t>
+          <t>ROSSY GONSALVES</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 00 Mins</t>
+          <t>00 Hrs 29 Mins</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>A.B.STEEL,LIMITADA</t>
+          <t>HAO FA COMERCIALL</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 00 Mins</t>
+          <t>00 Hrs 10 Mins</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>RICARDO DINIS LANGA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>KHAN FERRAGEM ELECTRICO, LDA</t>
+          <t>AGOSTINHO</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 00 Mins</t>
+          <t>00 Hrs 11 Mins</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SAIDATA ZALIA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>RAGE COMERCIAL</t>
+          <t>FERNEX</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 16 Mins</t>
+          <t>00 Hrs 10 Mins</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SAIDATA ZALIA</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>AMAL COMERCIAL</t>
+          <t>IMRANYAKUB</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 12 Mins</t>
+          <t>00 Hrs 16 Mins</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>AF FERRAGEM E.I</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 08 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>AUTO FERRAGEM PEQUENINO</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 39 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM MUHENGO, LDA</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>01 Hrs 01 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>FERRAGEM SERGIO E.I</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 45 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>RICARDO DINIS LANGA</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>FANTASTIC INDUSTRIES, LDA</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 00 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>SAIDATA ZALIA</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>CENTRO DE FERRAGEM</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 29 Mins</t>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>EMCO LDA</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 12 Mins</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>SAIDATA ZALIA</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>KHALID SU LDA</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>00 Hrs 10 Mins</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
must fear the env all times
</commit_message>
<xml_diff>
--- a/Daily_CSFA_Report.xlsx
+++ b/Daily_CSFA_Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance Grid - March" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Attendance - March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Visits" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Day Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Attendance Grid - March" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly Attendance - March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Day Visits" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <name val="Times New Roman"/>
@@ -82,22 +79,22 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -497,7 +494,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -512,7 +509,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -527,7 +524,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -572,7 +569,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -587,7 +584,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -602,7 +599,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -632,11 +629,11 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Used App</t>
+          <t>Did Not Use App</t>
         </is>
       </c>
     </row>
@@ -826,7 +823,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q2" s="5" t="inlineStr"/>
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr"/>
@@ -836,7 +837,7 @@
       <c r="W2" s="5" t="inlineStr"/>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>1/1 - Perfect attendance</t>
+          <t>2/2 - Perfect attendance</t>
         </is>
       </c>
     </row>
@@ -916,7 +917,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr"/>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q3" s="5" t="inlineStr"/>
       <c r="R3" s="5" t="inlineStr"/>
       <c r="S3" s="5" t="inlineStr"/>
@@ -926,7 +931,7 @@
       <c r="W3" s="5" t="inlineStr"/>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1011,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr"/>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q4" s="5" t="inlineStr"/>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr"/>
@@ -1016,7 +1025,7 @@
       <c r="W4" s="5" t="inlineStr"/>
       <c r="X4" s="5" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1105,11 @@
           <t>SUS</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr"/>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
       <c r="S5" s="5" t="inlineStr"/>
@@ -1186,7 +1199,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q6" s="5" t="inlineStr"/>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr"/>
@@ -1196,7 +1213,7 @@
       <c r="W6" s="5" t="inlineStr"/>
       <c r="X6" s="5" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1293,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P7" s="5" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q7" s="5" t="inlineStr"/>
       <c r="R7" s="5" t="inlineStr"/>
       <c r="S7" s="5" t="inlineStr"/>
@@ -1286,7 +1307,7 @@
       <c r="W7" s="5" t="inlineStr"/>
       <c r="X7" s="5" t="inlineStr">
         <is>
-          <t>14/14 - Perfect attendance</t>
+          <t>15/15 - Perfect attendance</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1387,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q8" s="5" t="inlineStr"/>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr"/>
@@ -1376,7 +1401,7 @@
       <c r="W8" s="5" t="inlineStr"/>
       <c r="X8" s="5" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1481,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P9" s="5" t="inlineStr"/>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q9" s="5" t="inlineStr"/>
       <c r="R9" s="5" t="inlineStr"/>
       <c r="S9" s="5" t="inlineStr"/>
@@ -1466,7 +1495,7 @@
       <c r="W9" s="5" t="inlineStr"/>
       <c r="X9" s="5" t="inlineStr">
         <is>
-          <t>14/14 - Perfect attendance</t>
+          <t>15/15 - Perfect attendance</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1575,11 @@
           <t>SUS</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr"/>
+      <c r="P10" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
       <c r="Q10" s="5" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr"/>
@@ -1636,7 +1669,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P11" s="5" t="inlineStr"/>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q11" s="5" t="inlineStr"/>
       <c r="R11" s="5" t="inlineStr"/>
       <c r="S11" s="5" t="inlineStr"/>
@@ -1646,7 +1683,7 @@
       <c r="W11" s="5" t="inlineStr"/>
       <c r="X11" s="5" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1765,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="25" customHeight="1">
+    <row r="6" ht="39.2" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>IMRAN AHMED</t>
@@ -1736,7 +1773,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>No attendance on dates: 4, 5, 6, 9, 11, 19 (6 days)</t>
+          <t>No attendance on dates: 4, 5, 6, 9, 11, 19, 20 (7 days)</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1833,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>No attendance on dates: 2, 3, 4, 13 (4 days)</t>
+          <t>No attendance on dates: 2, 3, 4, 13, 20 (5 days)</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1849,7 +1886,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 16 Mins</t>
+          <t>01 Hrs 02 Mins</t>
         </is>
       </c>
     </row>
@@ -1861,12 +1898,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>UAMUSSE FERRANGEM</t>
+          <t>FERRAGEM TAWAKULL</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 07 Mins</t>
+          <t>00 Hrs 24 Mins</t>
         </is>
       </c>
     </row>
@@ -1878,12 +1915,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM GLORIOSO</t>
+          <t>O.S HOLDING, LDA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 15 Mins</t>
+          <t>00 Hrs 18 Mins</t>
         </is>
       </c>
     </row>
@@ -1895,12 +1932,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ROYAL FERRAGEM SUCURSAL LDA</t>
+          <t>FERRAGENS JALASAI</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 10 Mins</t>
+          <t>00 Hrs 19 Mins</t>
         </is>
       </c>
     </row>
@@ -1912,12 +1949,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM UNIVERSAL</t>
+          <t>TINTAS E FERRAGENS, LDA</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 08 Mins</t>
+          <t>00 Hrs 10 Mins</t>
         </is>
       </c>
     </row>
@@ -1929,63 +1966,63 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>P.P. IMPORTACAO E EXPORTACAO</t>
+          <t>FERRAGEM SAMANTHA</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 08 Mins</t>
+          <t>00 Hrs 16 Mins</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ADERITO MACHOVO</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>LANGA COMERCIAL SOC UNP LDA</t>
+          <t>FERRAGEM EBENEZER</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 08 Mins</t>
+          <t>00 Hrs 18 Mins</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ADERITO MACHOVO</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM TENHA FÉ</t>
+          <t>FERRAGEM 1º DE MAIO</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 08 Mins</t>
+          <t>00 Hrs 28 Mins</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ADERITO MACHOVO</t>
+          <t>ANDRE MARQUEZA</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>TINTAS E FERRAGENS, LDA</t>
+          <t>FRANCIS FERRAGEM SOC. UNIP. LDA</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 07 Mins</t>
+          <t>00 Hrs 30 Mins</t>
         </is>
       </c>
     </row>
@@ -1997,12 +2034,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>MASSANGO PAINTS, EI</t>
+          <t>FERRAGEM BOM TEMPO</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 17 Mins</t>
+          <t>00 Hrs 34 Mins</t>
         </is>
       </c>
     </row>
@@ -2014,641 +2051,318 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM DAS MAHOTAS,LDA</t>
+          <t>KADI COMERCIAL</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 21 Mins</t>
+          <t>00 Hrs 32 Mins</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>QUATRO ESTRELAS FERRAGENS</t>
+          <t>FERRAGEM AFRIPAK TRADING EI</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 43 Mins</t>
+          <t>00 Hrs 14 Mins</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHINA MALL, LDA</t>
+          <t>ARIMEK COMERCIAL EI</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 30 Mins</t>
+          <t>00 Hrs 10 Mins</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>FRANCISCO TOMAS</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>KUSHI MAPUTO LDA</t>
+          <t>FERRAGEM AUTO GEMO</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 16 Mins</t>
+          <t>00 Hrs 06 Mins</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM PONTE, LDA</t>
+          <t>JKAS COMERCIAL, LDA</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 16 Mins</t>
+          <t>00 Hrs 02 Mins</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ANDRE MARQUEZA</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>LIMPOPO TRADING, LDA</t>
+          <t>ROMSHA TRADING, LDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 29 Mins</t>
+          <t>00 Hrs 03 Mins</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM CH CONSTRUCOES</t>
+          <t>INDO AFRICA COMERCIAL - ARMAZENS VITORIA</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 15 Mins</t>
+          <t>00 Hrs 07 Mins</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM SOBRINHO DE DEUS</t>
+          <t>KAAFERR FERRAGEM</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 08 Mins</t>
+          <t>00 Hrs 03 Mins</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PATEL HARDWARE MOCAMBIQUE</t>
+          <t>CONSTRUCTION SITE - AVENIDA MILAGRE MAPOTE</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 09 Mins</t>
+          <t>00 Hrs 07 Mins</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>ITO BENEDITO</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM RHUMBANE</t>
+          <t>FERRAGEM BAIANA</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 15 Mins</t>
+          <t>00 Hrs 07 Mins</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>FRANCISCO TOMAS</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>JIANGHAI CONSTRUCOES E SOCIEDADE UNIPESSOAL, LDA</t>
+          <t>G.F COMERCIAL</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 10 Mins</t>
+          <t>00 Hrs 06 Mins</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE BERTUR</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>KULUN MATERIAL DE CONSTRUCAO, LIMITADA</t>
+          <t>FERRAGEM L.H.A</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 25 Mins</t>
+          <t>00 Hrs 13 Mins</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE BERTUR</t>
+          <t>KUMAR CHAMPAKLAL</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>FERCON</t>
+          <t>LUA E MAR</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 24 Mins</t>
+          <t>00 Hrs 07 Mins</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE BERTUR</t>
+          <t>RICARDO DINIS LANGA</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM MAHAMCOMERCIAL</t>
+          <t>TINTAS BERGER MAPUTO OFFICE</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 02 Mins</t>
+          <t>00 Hrs 40 Mins</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE BERTUR</t>
+          <t>RICARDO DINIS LANGA</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ROSE GONSALVES</t>
+          <t>BEST CHAPA SOCIEDADE-UNIPESSOAL LDA</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 25 Mins</t>
+          <t>00 Hrs 40 Mins</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE BERTUR</t>
+          <t>RICARDO DINIS LANGA</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>HAO FA COMERCIAL</t>
+          <t>FERRAGEM MACICAME, SOCIEDADE UNIPESSOAL, LDA</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>01 Hrs 18 Mins</t>
+          <t>00 Hrs 25 Mins</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE BERTUR</t>
+          <t>RICARDO DINIS LANGA</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>FERNEX FERRAGEM</t>
+          <t>IFRESH, LDA</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 05 Mins</t>
+          <t>00 Hrs 22 Mins</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE BERTUR</t>
+          <t>RICARDO DINIS LANGA</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>IMRAN FERRAGEM</t>
+          <t>FERRAGEM NATAL</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 16 Mins</t>
+          <t>00 Hrs 12 Mins</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ITO BENEDITO</t>
+          <t>RICARDO DINIS LANGA</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>FERRAGEM AFRIPAK TRADING EI</t>
+          <t>FERRAGEM ALMADINA SOC.UNIP,LDA</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>00 Hrs 09 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>ITO BENEDITO</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>ARIMEK COMERCIAL EI</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 18 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>ITO BENEDITO</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>MODALAND INTERPRICES</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 09 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>ITO BENEDITO</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>GOD WIN FERRAGEM</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 06 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>ITO BENEDITO</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>FERRAGEM AUTO GEMO</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 05 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>ITO BENEDITO</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>MOBILITY INVESTIMENTO, EI</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 14 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>ITO BENEDITO</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>FERRAGEM PURE ON HEART</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 03 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>KUMAR CHAMPAKLAL</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>LUA E MAR</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 47 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>KUMAR CHAMPAKLAL</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>ROSSY GONSALVES</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 29 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>KUMAR CHAMPAKLAL</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>HAO FA COMERCIALL</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 10 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>KUMAR CHAMPAKLAL</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>AGOSTINHO</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 11 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>KUMAR CHAMPAKLAL</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>FERNEX</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 10 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>KUMAR CHAMPAKLAL</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>IMRANYAKUB</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 16 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>RICARDO DINIS LANGA</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>AF FERRAGEM E.I</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 08 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>RICARDO DINIS LANGA</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>AUTO FERRAGEM PEQUENINO</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 39 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>RICARDO DINIS LANGA</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>FERRAGEM MUHENGO, LDA</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>01 Hrs 01 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>RICARDO DINIS LANGA</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>FERRAGEM SERGIO E.I</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 45 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>RICARDO DINIS LANGA</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>FANTASTIC INDUSTRIES, LDA</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 00 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>SAIDATA ZALIA</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>EMCO LDA</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 12 Mins</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>SAIDATA ZALIA</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>KHALID SU LDA</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>00 Hrs 10 Mins</t>
+          <t>00 Hrs 27 Mins</t>
         </is>
       </c>
     </row>

</xml_diff>